<commit_message>
Update de Roteiro de Teste
Roteiro de Teste, testando todos os pontos apresentados
</commit_message>
<xml_diff>
--- a/4.Teste/0FUMO - Roteiro de Teste.xlsx
+++ b/4.Teste/0FUMO - Roteiro de Teste.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E303327\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aluno\Downloads\git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{532A4351-9001-48E3-B010-5E418E86CB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19170" yWindow="14270" windowWidth="21660" windowHeight="9440" tabRatio="913" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" tabRatio="913" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
@@ -23,7 +22,7 @@
     <definedName name="__xlfn_IFERROR">NA()</definedName>
     <definedName name="combo_SimNao">AUX!$A$2:$A$3</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -125,9 +124,6 @@
     <t>Nome, e-mail válido, senha válida</t>
   </si>
   <si>
-    <t>Usuário cadastrado com sucesso e redirecionado para avaliação inicial</t>
-  </si>
-  <si>
     <t>Validar campos obrigatórios</t>
   </si>
   <si>
@@ -183,12 +179,15 @@
   </si>
   <si>
     <t>Usuário não possuir cadastro no sistema e acessar a tela de cadastro.</t>
+  </si>
+  <si>
+    <t>Usuário cadastrado com sucesso</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -863,6 +862,15 @@
     <xf numFmtId="0" fontId="23" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="16" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -884,31 +892,22 @@
     <xf numFmtId="0" fontId="23" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="15">
-    <cellStyle name="Bom" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Bom" xfId="1"/>
     <cellStyle name="Cálculo" xfId="2" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Célula de Verificação" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Célula de Verificação" xfId="3"/>
     <cellStyle name="Entrada" xfId="4" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Neutra" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Incorreto" xfId="5" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Neutra" xfId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Normal 3" xfId="7"/>
     <cellStyle name="Nota" xfId="8" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Porcentagem 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Ruim" xfId="5" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Porcentagem 2" xfId="9"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="11" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="12" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título 5" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Título 5" xfId="13"/>
     <cellStyle name="Total" xfId="14" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1339,7 +1338,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:L22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1360,18 +1359,18 @@
     <row r="1" spans="2:12" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:12" ht="18.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="24"/>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="33"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="36"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B3" s="25"/>
@@ -1408,7 +1407,7 @@
         <v>7</v>
       </c>
       <c r="F5" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="20">
         <v>0</v>
@@ -1567,7 +1566,7 @@
       </c>
       <c r="F21" s="3">
         <f>SUM(F5:F19)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="3">
         <f>SUM(G5:G19)</f>
@@ -1579,7 +1578,7 @@
       </c>
       <c r="I21" s="27">
         <f>SUM(F21:H21)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="26"/>
     </row>
@@ -1608,7 +1607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1640,7 +1639,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1654,31 +1653,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
     </row>
     <row r="2" spans="1:23" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="35">
+      <c r="A2" s="38">
         <v>7</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
     </row>
     <row r="3" spans="1:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="38"/>
+      <c r="B4" s="41"/>
       <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -1694,7 +1693,7 @@
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1722,21 +1721,25 @@
       </c>
     </row>
     <row r="9" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A9" s="39">
+      <c r="A9" s="32">
         <v>1</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="41" t="s">
-        <v>27</v>
+      <c r="D9" s="34" t="s">
+        <v>46</v>
       </c>
       <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>1</v>
+      </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -1755,21 +1758,25 @@
       <c r="W9" s="5"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A10" s="40">
+      <c r="A10" s="33">
         <v>2</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="D10" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="41" t="s">
-        <v>30</v>
-      </c>
       <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <v>1</v>
+      </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -1788,92 +1795,112 @@
       <c r="W10" s="5"/>
     </row>
     <row r="11" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="40">
+      <c r="A11" s="33">
         <v>3</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="D11" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="E11" s="14"/>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A12" s="33">
+        <v>4</v>
+      </c>
+      <c r="B12" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-    </row>
-    <row r="12" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="40">
-        <v>4</v>
-      </c>
-      <c r="B12" s="41" t="s">
+      <c r="C12" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="41" t="s">
+      <c r="D12" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="E12" s="13"/>
+      <c r="F12" s="13">
+        <v>0</v>
+      </c>
+      <c r="G12" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="33">
+        <v>5</v>
+      </c>
+      <c r="B13" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="40">
-        <v>5</v>
-      </c>
-      <c r="B13" s="41" t="s">
+      <c r="C13" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="D13" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="E13" s="13"/>
+      <c r="F13" s="13">
+        <v>1</v>
+      </c>
+      <c r="G13" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="32">
+        <v>6</v>
+      </c>
+      <c r="B14" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="39">
-        <v>6</v>
-      </c>
-      <c r="B14" s="41" t="s">
+      <c r="C14" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="D14" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="E14" s="13"/>
+      <c r="F14" s="13">
+        <v>0</v>
+      </c>
+      <c r="G14" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A15" s="33">
+        <v>7</v>
+      </c>
+      <c r="B15" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="1:23" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A15" s="40">
-        <v>7</v>
-      </c>
-      <c r="B15" s="41" t="s">
+      <c r="C15" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="D15" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="41" t="s">
-        <v>45</v>
-      </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
+      <c r="F15" s="13">
+        <v>0</v>
+      </c>
+      <c r="G15" s="13">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="40">
+      <c r="A16" s="33">
         <v>8</v>
       </c>
       <c r="B16" s="6"/>
@@ -1884,7 +1911,7 @@
       <c r="G16" s="14"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="40">
+      <c r="A17" s="33">
         <v>9</v>
       </c>
       <c r="B17" s="6"/>
@@ -1895,7 +1922,7 @@
       <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="40">
+      <c r="A18" s="33">
         <v>10</v>
       </c>
       <c r="B18" s="6"/>
@@ -1906,7 +1933,7 @@
       <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="39">
+      <c r="A19" s="32">
         <v>11</v>
       </c>
       <c r="B19" s="11"/>
@@ -1934,7 +1961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1949,31 +1976,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
     </row>
     <row r="2" spans="1:23" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="35">
+      <c r="A2" s="38">
         <v>6</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
     </row>
     <row r="3" spans="1:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="38"/>
+      <c r="B4" s="41"/>
       <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:23" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>